<commit_message>
Better Prompting for Optimization suggs
</commit_message>
<xml_diff>
--- a/.files/Test_Report.xlsx
+++ b/.files/Test_Report.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00_-"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +46,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -161,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,6 +202,8 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1637,7 +1642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -3085,215 +3090,101 @@
       <c r="C42" s="26" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>Overhead Materials</t>
-        </is>
-      </c>
-      <c r="C43" s="18" t="n">
-        <v>36.930725</v>
-      </c>
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>(None configured)</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>Overhead Labor</t>
-        </is>
-      </c>
-      <c r="C44" s="18" t="n">
-        <v>36.930725</v>
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="n"/>
+      <c r="C44" s="31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="17" t="inlineStr">
-        <is>
-          <t>Admin and Management</t>
-        </is>
-      </c>
-      <c r="C45" s="18" t="n">
-        <v>36.930725</v>
-      </c>
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>MARKUPS / PROFIT</t>
+        </is>
+      </c>
+      <c r="B45" s="33" t="n"/>
+      <c r="C45" s="34" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="n">
-        <v>36.930725</v>
-      </c>
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>(None configured)</t>
+        </is>
+      </c>
+      <c r="C46" s="28" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>Packaging Materials</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="n">
-        <v>36.930725</v>
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B47" s="30" t="n"/>
+      <c r="C47" s="31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="inlineStr">
-        <is>
-          <t>Shipping and Transport</t>
-        </is>
-      </c>
-      <c r="C48" s="18" t="n">
-        <v>36.930725</v>
-      </c>
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>PROJECT TOTAL</t>
+        </is>
+      </c>
+      <c r="B48" s="36" t="n"/>
+      <c r="C48" s="37" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>Commissions</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="n">
-        <v>36.930725</v>
+      <c r="A49" s="38" t="inlineStr">
+        <is>
+          <t>Discounted Total:</t>
+        </is>
+      </c>
+      <c r="B49" s="39" t="n"/>
+      <c r="C49" s="40" t="n">
+        <v>3693.0725</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="inlineStr">
-        <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="B50" s="28" t="n"/>
-      <c r="C50" s="29" t="n">
-        <v>258.515075</v>
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>+ Miscellaneous:</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="30" t="inlineStr">
-        <is>
-          <t>MARKUPS / PROFIT</t>
-        </is>
-      </c>
-      <c r="B51" s="31" t="n"/>
-      <c r="C51" s="32" t="n"/>
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>+ Markups:</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="inlineStr">
-        <is>
-          <t>Profit on Material</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="n">
-        <v>24.536975</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>Profit on Waste</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="n">
-        <v>11.30844733333333</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="17" t="inlineStr">
-        <is>
-          <t>Profit on Glass Purchase</t>
-        </is>
-      </c>
-      <c r="C54" s="18" t="n">
-        <v>8.793750000000001</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>Profit on Wages</t>
-        </is>
-      </c>
-      <c r="C55" s="18" t="n">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="17" t="inlineStr">
-        <is>
-          <t>Planning / Technical Office</t>
-        </is>
-      </c>
-      <c r="C56" s="18" t="n">
-        <v>36.930725</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>Commission</t>
-        </is>
-      </c>
-      <c r="C57" s="18" t="n">
-        <v>36.930725</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="B58" s="28" t="n"/>
-      <c r="C58" s="29" t="n">
-        <v>122.1006223333333</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="33" t="inlineStr">
-        <is>
-          <t>PROJECT TOTAL</t>
-        </is>
-      </c>
-      <c r="B59" s="34" t="n"/>
-      <c r="C59" s="35" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="36" t="inlineStr">
-        <is>
-          <t>Discounted Total:</t>
-        </is>
-      </c>
-      <c r="B60" s="37" t="n"/>
-      <c r="C60" s="38" t="n">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL:</t>
+        </is>
+      </c>
+      <c r="B52" s="42" t="n"/>
+      <c r="C52" s="43" t="n">
         <v>3693.0725</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>+ Miscellaneous:</t>
-        </is>
-      </c>
-      <c r="C61" s="18" t="n">
-        <v>258.515075</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="17" t="inlineStr">
-        <is>
-          <t>+ Markups:</t>
-        </is>
-      </c>
-      <c r="C62" s="18" t="n">
-        <v>122.1006223333333</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="39" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL:</t>
-        </is>
-      </c>
-      <c r="B63" s="40" t="n"/>
-      <c r="C63" s="41" t="n">
-        <v>4073.688197333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>